<commit_message>
Updated ProductLifecycle.xlsx dates and product names for SQL and Windows, version currency for SQL
</commit_message>
<xml_diff>
--- a/ProductLifecycle.xlsx
+++ b/ProductLifecycle.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\azure-arc-dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26A228B9-0FFA-42A7-8EDD-F9FB34E716F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4499244-1E46-4170-8B7F-9F885A932B18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28965" yWindow="-165" windowWidth="29130" windowHeight="17610" xr2:uid="{F101B0D7-EE75-4F00-B8B9-EF6AEAB46F08}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{F101B0D7-EE75-4F00-B8B9-EF6AEAB46F08}"/>
   </bookViews>
   <sheets>
     <sheet name="ProductLifecycle" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ProductLifecycle!$A$1:$F$126</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ProductLifecycle!$A$1:$F$132</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="234">
   <si>
     <t>Amazon Linux 2</t>
   </si>
@@ -714,6 +714,30 @@
   </si>
   <si>
     <t>Ubuntu 22.04.3 LTS</t>
+  </si>
+  <si>
+    <t>SQL Server 2025 Developer</t>
+  </si>
+  <si>
+    <t>SQL Server 2025 Enterprise</t>
+  </si>
+  <si>
+    <t>SQL Server 2025 Evaluation</t>
+  </si>
+  <si>
+    <t>SQL Server 2025 Express</t>
+  </si>
+  <si>
+    <t>SQL Server 2025 Standard</t>
+  </si>
+  <si>
+    <t>https://learn.microsoft.com/en-us/lifecycle/products/sql-server-2025</t>
+  </si>
+  <si>
+    <t>N-6</t>
+  </si>
+  <si>
+    <t>Windows Server 2025 Standard</t>
   </si>
 </sst>
 </file>
@@ -1329,8 +1353,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2C44A62F-1B70-43DD-B7C4-B92B4D45F557}" name="ProductLifecycle" displayName="ProductLifecycle" ref="A1:L126" totalsRowShown="0" headerRowDxfId="8">
-  <autoFilter ref="A1:L126" xr:uid="{3B9240C1-6AC6-450B-B825-FF7619896A12}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2C44A62F-1B70-43DD-B7C4-B92B4D45F557}" name="ProductLifecycle" displayName="ProductLifecycle" ref="A1:L132" totalsRowShown="0" headerRowDxfId="8">
+  <autoFilter ref="A1:L132" xr:uid="{3B9240C1-6AC6-450B-B825-FF7619896A12}"/>
   <tableColumns count="12">
     <tableColumn id="1" xr3:uid="{03DD380E-4CBD-4AF4-A333-BBB151740B8A}" name="Product"/>
     <tableColumn id="8" xr3:uid="{40F3BF2C-2608-4F0E-9DA8-4D12D683F91C}" name="ProductFriendlyName"/>
@@ -1666,7 +1690,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B9240C1-6AC6-450B-B825-FF7619896A12}">
-  <dimension ref="A1:L126"/>
+  <dimension ref="A1:L132"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="70.26953125" customWidth="1"/>
@@ -1678,7 +1702,7 @@
     <col min="7" max="7" width="38.7265625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="20.54296875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20.26953125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="85.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="59.26953125" customWidth="1"/>
     <col min="11" max="11" width="16.1796875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="21.08984375" bestFit="1" customWidth="1"/>
   </cols>
@@ -2859,7 +2883,7 @@
         <v>0</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.35">
@@ -2895,7 +2919,7 @@
         <v>0</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.35">
@@ -2933,7 +2957,7 @@
         <v>0</v>
       </c>
       <c r="L41" s="1" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.35">
@@ -2971,7 +2995,7 @@
         <v>0</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.35">
@@ -3007,7 +3031,7 @@
         <v>0</v>
       </c>
       <c r="L43" s="1" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.35">
@@ -3045,7 +3069,7 @@
         <v>0</v>
       </c>
       <c r="L44" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.35">
@@ -3083,7 +3107,7 @@
         <v>0</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.35">
@@ -3121,7 +3145,7 @@
         <v>0</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.35">
@@ -3159,7 +3183,7 @@
         <v>0</v>
       </c>
       <c r="L47" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.35">
@@ -3197,7 +3221,7 @@
         <v>0</v>
       </c>
       <c r="L48" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.35">
@@ -3217,7 +3241,7 @@
         <v>46187</v>
       </c>
       <c r="F49" s="1">
-        <v>47283</v>
+        <v>47316</v>
       </c>
       <c r="G49" s="3">
         <v>139</v>
@@ -3235,7 +3259,7 @@
         <v>1</v>
       </c>
       <c r="L49" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.35">
@@ -3255,7 +3279,7 @@
         <v>46187</v>
       </c>
       <c r="F50" s="1">
-        <v>47283</v>
+        <v>47316</v>
       </c>
       <c r="G50" s="3">
         <v>139</v>
@@ -3273,7 +3297,7 @@
         <v>1</v>
       </c>
       <c r="L50" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.35">
@@ -3293,7 +3317,7 @@
         <v>46217</v>
       </c>
       <c r="F51" s="1">
-        <v>47313</v>
+        <v>47316</v>
       </c>
       <c r="G51" s="3">
         <v>0</v>
@@ -3311,7 +3335,7 @@
         <v>0</v>
       </c>
       <c r="L51" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.35">
@@ -3331,7 +3355,7 @@
         <v>46217</v>
       </c>
       <c r="F52" s="1">
-        <v>47313</v>
+        <v>47316</v>
       </c>
       <c r="G52" s="3">
         <v>540.5</v>
@@ -3349,7 +3373,7 @@
         <v>0</v>
       </c>
       <c r="L52" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.35">
@@ -3369,7 +3393,7 @@
         <v>46217</v>
       </c>
       <c r="F53" s="1">
-        <v>47313</v>
+        <v>47316</v>
       </c>
       <c r="G53" s="3">
         <v>0</v>
@@ -3387,7 +3411,7 @@
         <v>0</v>
       </c>
       <c r="L53" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.35">
@@ -3407,7 +3431,7 @@
         <v>46217</v>
       </c>
       <c r="F54" s="1">
-        <v>47313</v>
+        <v>47316</v>
       </c>
       <c r="G54" s="3">
         <v>0</v>
@@ -3425,7 +3449,7 @@
         <v>0</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.35">
@@ -3445,7 +3469,7 @@
         <v>46217</v>
       </c>
       <c r="F55" s="1">
-        <v>47313</v>
+        <v>47316</v>
       </c>
       <c r="G55" s="3">
         <v>139</v>
@@ -3463,7 +3487,7 @@
         <v>0</v>
       </c>
       <c r="L55" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.35">
@@ -3483,7 +3507,7 @@
         <v>46672</v>
       </c>
       <c r="F56" s="1">
-        <v>47768</v>
+        <v>46672</v>
       </c>
       <c r="G56" s="3"/>
       <c r="H56" s="1" t="b">
@@ -3499,7 +3523,7 @@
         <v>1</v>
       </c>
       <c r="L56" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.35">
@@ -3519,7 +3543,7 @@
         <v>46672</v>
       </c>
       <c r="F57" s="1">
-        <v>47768</v>
+        <v>46672</v>
       </c>
       <c r="G57" s="3"/>
       <c r="H57" s="1" t="b">
@@ -3535,7 +3559,7 @@
         <v>1</v>
       </c>
       <c r="L57" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.35">
@@ -3555,11 +3579,9 @@
         <v>46672</v>
       </c>
       <c r="F58" s="1">
-        <v>47768</v>
-      </c>
-      <c r="G58" s="3">
-        <v>0</v>
-      </c>
+        <v>46672</v>
+      </c>
+      <c r="G58" s="3"/>
       <c r="H58" s="1" t="b">
         <v>1</v>
       </c>
@@ -3573,7 +3595,7 @@
         <v>0</v>
       </c>
       <c r="L58" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.35">
@@ -3593,7 +3615,7 @@
         <v>46672</v>
       </c>
       <c r="F59" s="1">
-        <v>47768</v>
+        <v>46672</v>
       </c>
       <c r="G59" s="3"/>
       <c r="H59" s="1" t="b">
@@ -3609,7 +3631,7 @@
         <v>0</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.35">
@@ -3629,11 +3651,9 @@
         <v>46672</v>
       </c>
       <c r="F60" s="1">
-        <v>47768</v>
-      </c>
-      <c r="G60" s="3">
-        <v>0</v>
-      </c>
+        <v>46672</v>
+      </c>
+      <c r="G60" s="3"/>
       <c r="H60" s="1" t="b">
         <v>0</v>
       </c>
@@ -3647,7 +3667,7 @@
         <v>0</v>
       </c>
       <c r="L60" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.35">
@@ -3667,11 +3687,9 @@
         <v>46672</v>
       </c>
       <c r="F61" s="1">
-        <v>47768</v>
-      </c>
-      <c r="G61" s="3">
-        <v>0</v>
-      </c>
+        <v>46672</v>
+      </c>
+      <c r="G61" s="3"/>
       <c r="H61" s="1" t="b">
         <v>1</v>
       </c>
@@ -3685,7 +3703,7 @@
         <v>0</v>
       </c>
       <c r="L61" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.35">
@@ -3705,7 +3723,7 @@
         <v>46672</v>
       </c>
       <c r="F62" s="1">
-        <v>47768</v>
+        <v>46672</v>
       </c>
       <c r="G62" s="3"/>
       <c r="H62" s="1" t="b">
@@ -3721,7 +3739,7 @@
         <v>0</v>
       </c>
       <c r="L62" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.35">
@@ -3757,7 +3775,7 @@
         <v>1</v>
       </c>
       <c r="L63" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.35">
@@ -3793,7 +3811,7 @@
         <v>1</v>
       </c>
       <c r="L64" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.35">
@@ -3815,9 +3833,7 @@
       <c r="F65" s="1">
         <v>48587</v>
       </c>
-      <c r="G65" s="3">
-        <v>0</v>
-      </c>
+      <c r="G65" s="3"/>
       <c r="H65" s="1" t="b">
         <v>1</v>
       </c>
@@ -3831,7 +3847,7 @@
         <v>0</v>
       </c>
       <c r="L65" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.35">
@@ -3867,7 +3883,7 @@
         <v>0</v>
       </c>
       <c r="L66" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.35">
@@ -3889,9 +3905,7 @@
       <c r="F67" s="1">
         <v>48587</v>
       </c>
-      <c r="G67" s="3">
-        <v>0</v>
-      </c>
+      <c r="G67" s="3"/>
       <c r="H67" s="1" t="b">
         <v>0</v>
       </c>
@@ -3905,7 +3919,7 @@
         <v>0</v>
       </c>
       <c r="L67" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.35">
@@ -3927,9 +3941,7 @@
       <c r="F68" s="1">
         <v>48587</v>
       </c>
-      <c r="G68" s="3">
-        <v>0</v>
-      </c>
+      <c r="G68" s="3"/>
       <c r="H68" s="1" t="b">
         <v>1</v>
       </c>
@@ -3943,7 +3955,7 @@
         <v>0</v>
       </c>
       <c r="L68" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.35">
@@ -3979,7 +3991,7 @@
         <v>0</v>
       </c>
       <c r="L69" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.35">
@@ -3999,7 +4011,7 @@
         <v>48590</v>
       </c>
       <c r="F70" s="1">
-        <v>49685</v>
+        <v>48590</v>
       </c>
       <c r="G70" s="3"/>
       <c r="H70" s="1" t="b">
@@ -4015,7 +4027,7 @@
         <v>1</v>
       </c>
       <c r="L70" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.35">
@@ -4035,11 +4047,9 @@
         <v>48590</v>
       </c>
       <c r="F71" s="1">
-        <v>49685</v>
-      </c>
-      <c r="G71" s="3">
-        <v>0</v>
-      </c>
+        <v>48590</v>
+      </c>
+      <c r="G71" s="3"/>
       <c r="H71" s="1" t="b">
         <v>1</v>
       </c>
@@ -4053,7 +4063,7 @@
         <v>0</v>
       </c>
       <c r="L71" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.35">
@@ -4073,7 +4083,7 @@
         <v>48590</v>
       </c>
       <c r="F72" s="1">
-        <v>49685</v>
+        <v>48590</v>
       </c>
       <c r="G72" s="3"/>
       <c r="H72" s="1" t="b">
@@ -4089,7 +4099,7 @@
         <v>0</v>
       </c>
       <c r="L72" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.35">
@@ -4109,11 +4119,9 @@
         <v>48590</v>
       </c>
       <c r="F73" s="1">
-        <v>49685</v>
-      </c>
-      <c r="G73" s="3">
-        <v>0</v>
-      </c>
+        <v>48590</v>
+      </c>
+      <c r="G73" s="3"/>
       <c r="H73" s="1" t="b">
         <v>1</v>
       </c>
@@ -4127,7 +4135,7 @@
         <v>0</v>
       </c>
       <c r="L73" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.35">
@@ -4147,11 +4155,9 @@
         <v>48590</v>
       </c>
       <c r="F74" s="1">
-        <v>49685</v>
-      </c>
-      <c r="G74" s="3">
-        <v>0</v>
-      </c>
+        <v>48590</v>
+      </c>
+      <c r="G74" s="3"/>
       <c r="H74" s="1" t="b">
         <v>1</v>
       </c>
@@ -4165,7 +4171,7 @@
         <v>0</v>
       </c>
       <c r="L74" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.35">
@@ -4185,7 +4191,7 @@
         <v>48590</v>
       </c>
       <c r="F75" s="1">
-        <v>49685</v>
+        <v>48590</v>
       </c>
       <c r="G75" s="3"/>
       <c r="H75" s="1" t="b">
@@ -4201,7 +4207,7 @@
         <v>0</v>
       </c>
       <c r="L75" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.35">
@@ -5941,7 +5947,7 @@
         <v>46399</v>
       </c>
       <c r="F126" s="1">
-        <v>46399</v>
+        <v>47494</v>
       </c>
       <c r="G126" s="3"/>
       <c r="H126" s="1" t="b">
@@ -5958,6 +5964,222 @@
       </c>
       <c r="L126" s="1" t="s">
         <v>219</v>
+      </c>
+    </row>
+    <row r="127" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A127" t="s">
+        <v>226</v>
+      </c>
+      <c r="B127" t="s">
+        <v>226</v>
+      </c>
+      <c r="C127" t="s">
+        <v>39</v>
+      </c>
+      <c r="D127" s="1">
+        <v>47854</v>
+      </c>
+      <c r="E127" s="1">
+        <v>49680</v>
+      </c>
+      <c r="F127" s="1">
+        <v>49680</v>
+      </c>
+      <c r="G127" s="3"/>
+      <c r="H127" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I127" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J127" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="K127" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L127" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="128" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A128" t="s">
+        <v>227</v>
+      </c>
+      <c r="B128" t="s">
+        <v>227</v>
+      </c>
+      <c r="C128" t="s">
+        <v>39</v>
+      </c>
+      <c r="D128" s="1">
+        <v>47854</v>
+      </c>
+      <c r="E128" s="1">
+        <v>49680</v>
+      </c>
+      <c r="F128" s="1">
+        <v>49680</v>
+      </c>
+      <c r="G128" s="3"/>
+      <c r="H128" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I128" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J128" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="K128" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L128" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="129" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A129" t="s">
+        <v>228</v>
+      </c>
+      <c r="B129" t="s">
+        <v>228</v>
+      </c>
+      <c r="C129" t="s">
+        <v>39</v>
+      </c>
+      <c r="D129" s="1">
+        <v>47854</v>
+      </c>
+      <c r="E129" s="1">
+        <v>49680</v>
+      </c>
+      <c r="F129" s="1">
+        <v>49680</v>
+      </c>
+      <c r="G129" s="3"/>
+      <c r="H129" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I129" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J129" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="K129" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L129" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="130" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A130" t="s">
+        <v>229</v>
+      </c>
+      <c r="B130" t="s">
+        <v>229</v>
+      </c>
+      <c r="C130" t="s">
+        <v>39</v>
+      </c>
+      <c r="D130" s="1">
+        <v>47854</v>
+      </c>
+      <c r="E130" s="1">
+        <v>49680</v>
+      </c>
+      <c r="F130" s="1">
+        <v>49680</v>
+      </c>
+      <c r="G130" s="3"/>
+      <c r="H130" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I130" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J130" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="K130" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L130" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="131" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A131" t="s">
+        <v>230</v>
+      </c>
+      <c r="B131" t="s">
+        <v>230</v>
+      </c>
+      <c r="C131" t="s">
+        <v>39</v>
+      </c>
+      <c r="D131" s="1">
+        <v>47854</v>
+      </c>
+      <c r="E131" s="1">
+        <v>49680</v>
+      </c>
+      <c r="F131" s="1">
+        <v>49680</v>
+      </c>
+      <c r="G131" s="3"/>
+      <c r="H131" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I131" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J131" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="K131" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L131" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="132" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A132" t="s">
+        <v>233</v>
+      </c>
+      <c r="B132" t="s">
+        <v>182</v>
+      </c>
+      <c r="C132" t="s">
+        <v>47</v>
+      </c>
+      <c r="D132" s="1">
+        <v>47435</v>
+      </c>
+      <c r="E132" s="1">
+        <v>49262</v>
+      </c>
+      <c r="F132" s="1">
+        <v>49262</v>
+      </c>
+      <c r="G132" s="3"/>
+      <c r="H132" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="I132" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="J132" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="K132" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="L132" s="1" t="s">
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -6016,10 +6238,11 @@
     <hyperlink ref="J49" r:id="rId51" xr:uid="{28F31A1E-41C9-4DA3-9278-4B6BA4E456F3}"/>
     <hyperlink ref="J56" r:id="rId52" xr:uid="{B86EF947-7BA1-45A9-BD8D-B9292A030200}"/>
     <hyperlink ref="J124" r:id="rId53" xr:uid="{6FCCDE1D-7AB1-4A22-9B61-AF173EAB6702}"/>
+    <hyperlink ref="J132" r:id="rId54" xr:uid="{16081F3F-9C57-4A8D-937E-8B769D78AA92}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId54"/>
+    <tablePart r:id="rId55"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>